<commit_message>
added doctor and turnout variable to 0th model of tisza
plus removed unnecessary files
</commit_message>
<xml_diff>
--- a/data/description.xlsx
+++ b/data/description.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10215"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac/Downloads/egyetem/TDK/magyar_petered_main/magyar_petered/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5F14167-FECA-124A-B84D-061CA54975D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4E78A39-C694-8944-BC6A-0E54F5439938}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="120">
   <si>
     <t>name</t>
   </si>
@@ -388,6 +388,12 @@
   </si>
   <si>
     <t>Népesség</t>
+  </si>
+  <si>
+    <t>doctor</t>
+  </si>
+  <si>
+    <t>Egy háziorvosra jutó évi betegforgalom</t>
   </si>
 </sst>
 </file>
@@ -777,7 +783,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E7187CE-9F21-A342-8F7F-7ACF8D8CCA35}">
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.6640625" style="3" bestFit="1" customWidth="1"/>
@@ -975,29 +981,29 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A12" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>51</v>
+    <row r="12" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>70</v>
       </c>
       <c r="E12" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>50</v>
@@ -1006,15 +1012,15 @@
         <v>51</v>
       </c>
       <c r="E13" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>50</v>
@@ -1028,16 +1034,16 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>50</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="E15" s="3">
         <v>1</v>
@@ -1045,10 +1051,10 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>50</v>
@@ -1062,16 +1068,16 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>50</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="E17" s="3">
         <v>1</v>
@@ -1079,16 +1085,16 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>50</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>57</v>
+        <v>70</v>
       </c>
       <c r="E18" s="3">
         <v>1</v>
@@ -1096,10 +1102,10 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>50</v>
@@ -1113,10 +1119,10 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>50</v>
@@ -1130,16 +1136,16 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>50</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="E21" s="3">
         <v>1</v>
@@ -1147,16 +1153,16 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>50</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E22" s="3">
         <v>1</v>
@@ -1164,33 +1170,33 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>50</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>70</v>
+        <v>53</v>
       </c>
       <c r="E23" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>102</v>
+        <v>22</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>50</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>57</v>
+        <v>70</v>
       </c>
       <c r="E24" s="3">
         <v>0</v>
@@ -1198,27 +1204,27 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>23</v>
+        <v>102</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>50</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="E25" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>50</v>
@@ -1226,33 +1232,33 @@
       <c r="D26" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="E26" s="4">
-        <v>0</v>
+      <c r="E26" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>50</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="E27" s="3">
-        <v>1</v>
+        <v>51</v>
+      </c>
+      <c r="E27" s="4">
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>50</v>
@@ -1261,55 +1267,55 @@
         <v>70</v>
       </c>
       <c r="E28" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
-        <v>27</v>
+        <v>81</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>82</v>
+        <v>26</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>50</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="E29" s="4">
+        <v>70</v>
+      </c>
+      <c r="E29" s="3">
         <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>50</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="E30" s="5">
+        <v>51</v>
+      </c>
+      <c r="E30" s="4">
         <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>50</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>51</v>
+        <v>70</v>
       </c>
       <c r="E31" s="5">
         <v>0</v>
@@ -1317,27 +1323,27 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
-        <v>85</v>
+        <v>29</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>30</v>
+        <v>84</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>86</v>
+        <v>50</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="E32" s="3">
+        <v>51</v>
+      </c>
+      <c r="E32" s="5">
         <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>86</v>
@@ -1351,10 +1357,10 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>86</v>
@@ -1368,10 +1374,10 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>86</v>
@@ -1385,10 +1391,10 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>86</v>
@@ -1402,10 +1408,10 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>86</v>
@@ -1419,10 +1425,10 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>86</v>
@@ -1436,10 +1442,10 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>86</v>
@@ -1453,10 +1459,10 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>86</v>
@@ -1470,10 +1476,10 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>86</v>
@@ -1487,10 +1493,10 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>86</v>
@@ -1504,10 +1510,10 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C43" s="2" t="s">
         <v>86</v>
@@ -1521,10 +1527,10 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C44" s="2" t="s">
         <v>86</v>
@@ -1538,10 +1544,10 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>86</v>
@@ -1555,44 +1561,44 @@
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="E46" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A47" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="B46" s="2" t="s">
+      <c r="B47" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C46" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="E46" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A47" s="3" t="s">
+      <c r="C47" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="E47" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+      <c r="A48" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="B47" s="6" t="s">
+      <c r="B48" s="6" t="s">
         <v>104</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="D47" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="E47" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A48" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="B48" s="3" t="s">
-        <v>105</v>
       </c>
       <c r="C48" s="2" t="s">
         <v>86</v>
@@ -1606,10 +1612,10 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A49" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C49" s="2" t="s">
         <v>86</v>
@@ -1623,10 +1629,10 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A50" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="C50" s="2" t="s">
         <v>86</v>
@@ -1640,10 +1646,10 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A51" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C51" s="2" t="s">
         <v>86</v>
@@ -1657,10 +1663,10 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A52" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C52" s="2" t="s">
         <v>86</v>
@@ -1674,10 +1680,10 @@
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A53" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C53" s="2" t="s">
         <v>86</v>
@@ -1691,18 +1697,35 @@
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A54" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="E54" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A55" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B54" s="3" t="s">
+      <c r="B55" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="C54" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="D54" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="E54" s="3">
+      <c r="C55" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="E55" s="3">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
rewrite models for pop.log1p
</commit_message>
<xml_diff>
--- a/data/description.xlsx
+++ b/data/description.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac/Downloads/egyetem/TDK/magyar_petered_main/magyar_petered/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4E78A39-C694-8944-BC6A-0E54F5439938}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA2A517B-628B-4540-9510-FE29B91E59CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -393,7 +393,7 @@
     <t>doctor</t>
   </si>
   <si>
-    <t>Egy háziorvosra jutó évi betegforgalom</t>
+    <t>Egy háziorvosra jutó évi betegforgalom_2024.csv</t>
   </si>
 </sst>
 </file>
@@ -1726,7 +1726,7 @@
         <v>70</v>
       </c>
       <c r="E55" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>